<commit_message>
KKT quote v3: uniform 8% profit, amounts derived from cost basis instead of targets
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014v4o941zghHSMa9tRzfaqP
</commit_message>
<xml_diff>
--- a/experiments/2026-10-12-kkt-drying-furnace-base/estimate/견적서_금강변압기_진공건조로_회전안착_용접_v3.xlsx
+++ b/experiments/2026-10-12-kkt-drying-furnace-base/estimate/견적서_금강변압기_진공건조로_회전안착_용접_v3.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="366">
   <si>
     <t xml:space="preserve">견          적          서</t>
   </si>
@@ -597,7 +597,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">일금 칠천오백일십육만팔백원정</t>
+    <t xml:space="preserve">일금 칠천오백칠십사만구천삼백원정</t>
   </si>
   <si>
     <t xml:space="preserve">No</t>
@@ -7630,7 +7630,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">) × 3.5%</t>
+      <t xml:space="preserve">) × 8.0%</t>
     </r>
   </si>
   <si>
@@ -8357,75 +8357,6 @@
   <si>
     <r>
       <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">노무비 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">+ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">경비 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">+ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">일반관리비</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) × 12.5%</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
         <b val="true"/>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -8648,75 +8579,6 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">3</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">노무비 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">+ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">경비 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">+ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">일반관리비</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) × 3.0%</t>
     </r>
   </si>
   <si>
@@ -12832,7 +12694,7 @@
       <c r="F16" s="12"/>
       <c r="G16" s="13" t="n">
         <f aca="false">원가계산서!E18</f>
-        <v>75160800</v>
+        <v>75749300</v>
       </c>
       <c r="H16" s="13"/>
       <c r="I16" s="13"/>
@@ -12878,7 +12740,7 @@
       </c>
       <c r="H19" s="18" t="n">
         <f aca="false">도비!$G$33</f>
-        <v>24213000</v>
+        <v>25206000</v>
       </c>
       <c r="I19" s="8" t="s">
         <v>41</v>
@@ -12902,7 +12764,7 @@
       </c>
       <c r="H20" s="18" t="n">
         <f aca="false">용접!$G$31</f>
-        <v>25653000</v>
+        <v>24747000</v>
       </c>
       <c r="I20" s="8" t="s">
         <v>45</v>
@@ -12926,7 +12788,7 @@
       </c>
       <c r="H21" s="18" t="n">
         <f aca="false">베이스!$G$34</f>
-        <v>18462000</v>
+        <v>18910000</v>
       </c>
       <c r="I21" s="8" t="s">
         <v>49</v>
@@ -12944,7 +12806,7 @@
       <c r="G22" s="3"/>
       <c r="H22" s="19" t="n">
         <f aca="false">SUM(H19:H21)</f>
-        <v>68328000</v>
+        <v>68863000</v>
       </c>
       <c r="I22" s="20"/>
     </row>
@@ -12960,7 +12822,7 @@
       <c r="G23" s="3"/>
       <c r="H23" s="19" t="n">
         <f aca="false">H22*0.1</f>
-        <v>6832800</v>
+        <v>6886300</v>
       </c>
       <c r="I23" s="20"/>
     </row>
@@ -12976,7 +12838,7 @@
       <c r="G24" s="21"/>
       <c r="H24" s="22" t="n">
         <f aca="false">H22+H23</f>
-        <v>75160800</v>
+        <v>75749300</v>
       </c>
       <c r="I24" s="7"/>
     </row>
@@ -13199,7 +13061,7 @@
       </c>
       <c r="F6" s="30" t="n">
         <f aca="false">E6/$E$16</f>
-        <v>0.19924042852125</v>
+        <v>0.197692519930877</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13224,7 +13086,7 @@
       </c>
       <c r="F7" s="30" t="n">
         <f aca="false">E7/$E$16</f>
-        <v>0.312756117550638</v>
+        <v>0.310326300045017</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13249,7 +13111,7 @@
       </c>
       <c r="F8" s="30" t="n">
         <f aca="false">E8/$E$16</f>
-        <v>0.360165671467041</v>
+        <v>0.357367526828631</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13274,7 +13136,7 @@
       </c>
       <c r="F9" s="30" t="n">
         <f aca="false">E9/$E$16</f>
-        <v>0.0111341177848027</v>
+        <v>0.0110476162816026</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13299,7 +13161,7 @@
       </c>
       <c r="F10" s="30" t="n">
         <f aca="false">E10/$E$16</f>
-        <v>0.00359669535183234</v>
+        <v>0.00356875245051769</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13324,7 +13186,7 @@
       </c>
       <c r="F11" s="30" t="n">
         <f aca="false">E11/$E$16</f>
-        <v>0.0159230925828357</v>
+        <v>0.0157993853012503</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13349,7 +13211,7 @@
       </c>
       <c r="F12" s="32" t="n">
         <f aca="false">E12/$E$16</f>
-        <v>0.902816123258401</v>
+        <v>0.895802100837896</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13374,7 +13236,7 @@
       </c>
       <c r="F13" s="30" t="n">
         <f aca="false">E13/$E$16</f>
-        <v>0.04514080616292</v>
+        <v>0.0447901050418948</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13383,23 +13245,23 @@
       </c>
       <c r="B14" s="18" t="n">
         <f aca="false">도비!$G$31</f>
-        <v>772159.5525</v>
+        <v>1764936.12</v>
       </c>
       <c r="C14" s="18" t="n">
         <f aca="false">용접!$G$29</f>
-        <v>2517017.8875</v>
+        <v>1610891.448</v>
       </c>
       <c r="D14" s="18" t="n">
         <f aca="false">베이스!$G$32</f>
-        <v>268813.694205</v>
+        <v>716836.51788</v>
       </c>
       <c r="E14" s="29" t="n">
         <f aca="false">SUM(B14:D14)</f>
-        <v>3557991.134205</v>
+        <v>4092664.08588</v>
       </c>
       <c r="F14" s="30" t="n">
         <f aca="false">E14/$E$16</f>
-        <v>0.0520722271134089</v>
+        <v>0.0594319748759131</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13408,23 +13270,23 @@
       </c>
       <c r="B15" s="18" t="n">
         <f aca="false">도비!$G$32</f>
-        <v>-861.052499998361</v>
+        <v>-637.620000001043</v>
       </c>
       <c r="C15" s="18" t="n">
         <f aca="false">용접!$G$30</f>
-        <v>-160.987500000745</v>
+        <v>-34.5480000004172</v>
       </c>
       <c r="D15" s="18" t="n">
         <f aca="false">베이스!$G$33</f>
-        <v>-970.167704999447</v>
+        <v>-992.991379998624</v>
       </c>
       <c r="E15" s="29" t="n">
         <f aca="false">SUM(B15:D15)</f>
-        <v>-1992.20770499855</v>
+        <v>-1665.15938000008</v>
       </c>
       <c r="F15" s="30" t="n">
         <f aca="false">E15/$E$16</f>
-        <v>-2.91565347295187E-005</v>
+        <v>-2.41807557033543E-005</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13433,19 +13295,19 @@
       </c>
       <c r="B16" s="31" t="n">
         <f aca="false">도비!$G$33</f>
-        <v>24213000</v>
+        <v>25206000</v>
       </c>
       <c r="C16" s="31" t="n">
         <f aca="false">용접!$G$31</f>
-        <v>25653000</v>
+        <v>24747000</v>
       </c>
       <c r="D16" s="31" t="n">
         <f aca="false">베이스!$G$34</f>
-        <v>18462000</v>
+        <v>18910000</v>
       </c>
       <c r="E16" s="19" t="n">
         <f aca="false">SUM(B16:D16)</f>
-        <v>68328000</v>
+        <v>68863000</v>
       </c>
       <c r="F16" s="32" t="n">
         <f aca="false">E16/$E$16</f>
@@ -13461,7 +13323,7 @@
       <c r="D17" s="33"/>
       <c r="E17" s="33" t="n">
         <f aca="false">E16*0.1</f>
-        <v>6832800</v>
+        <v>6886300</v>
       </c>
       <c r="F17" s="33"/>
     </row>
@@ -13474,7 +13336,7 @@
       <c r="D18" s="22"/>
       <c r="E18" s="22" t="n">
         <f aca="false">E16+E17</f>
-        <v>75160800</v>
+        <v>75749300</v>
       </c>
       <c r="F18" s="22"/>
     </row>
@@ -13899,7 +13761,7 @@
       <c r="D20" s="20"/>
       <c r="E20" s="39" t="n">
         <f aca="false">도비!$G$33-SUM(도비!$G$23:$G$25)</f>
-        <v>2568600</v>
+        <v>3561600</v>
       </c>
       <c r="F20" s="40" t="s">
         <v>141</v>
@@ -13915,7 +13777,7 @@
       <c r="D21" s="20"/>
       <c r="E21" s="39" t="n">
         <f aca="false">도비!$G$33</f>
-        <v>24213000</v>
+        <v>25206000</v>
       </c>
       <c r="F21" s="40" t="s">
         <v>143</v>
@@ -14227,7 +14089,7 @@
       <c r="D36" s="20"/>
       <c r="E36" s="39" t="n">
         <f aca="false">용접!$G$31-SUM(용접!$G$21:$G$23)</f>
-        <v>4393000</v>
+        <v>3487000</v>
       </c>
       <c r="F36" s="40" t="s">
         <v>141</v>
@@ -14243,7 +14105,7 @@
       <c r="D37" s="20"/>
       <c r="E37" s="39" t="n">
         <f aca="false">용접!$G$31</f>
-        <v>25653000</v>
+        <v>24747000</v>
       </c>
       <c r="F37" s="40" t="s">
         <v>178</v>
@@ -14615,7 +14477,7 @@
       <c r="D55" s="20"/>
       <c r="E55" s="39" t="n">
         <f aca="false">베이스!$G$34-SUM(베이스!$G$24:$G$26)</f>
-        <v>1773300</v>
+        <v>2221300</v>
       </c>
       <c r="F55" s="40" t="s">
         <v>141</v>
@@ -14631,7 +14493,7 @@
       <c r="D56" s="20"/>
       <c r="E56" s="39" t="n">
         <f aca="false">베이스!$G$34</f>
-        <v>18462000</v>
+        <v>18910000</v>
       </c>
       <c r="F56" s="40" t="s">
         <v>212</v>
@@ -15323,7 +15185,7 @@
       <c r="F31" s="43"/>
       <c r="G31" s="44" t="n">
         <f aca="false">(G24+G25+G26+G27+G28+G30)*요율근거!$C$9</f>
-        <v>772159.5525</v>
+        <v>1764936.12</v>
       </c>
       <c r="H31" s="20" t="s">
         <v>246</v>
@@ -15341,7 +15203,7 @@
       <c r="F32" s="43"/>
       <c r="G32" s="44" t="n">
         <f aca="false">-MOD(G29+G30+G31,1000)</f>
-        <v>-861.052499998361</v>
+        <v>-637.620000001043</v>
       </c>
       <c r="H32" s="40" t="s">
         <v>247</v>
@@ -15359,7 +15221,7 @@
       <c r="F33" s="45"/>
       <c r="G33" s="46" t="n">
         <f aca="false">G29+G30+G31+G32</f>
-        <v>24213000</v>
+        <v>25206000</v>
       </c>
       <c r="H33" s="10" t="s">
         <v>248</v>
@@ -16049,10 +15911,10 @@
       <c r="F29" s="43"/>
       <c r="G29" s="44" t="n">
         <f aca="false">(G22+G23+G24+G25+G26+G28)*요율근거!$C$10</f>
-        <v>2517017.8875</v>
+        <v>1610891.448</v>
       </c>
       <c r="H29" s="20" t="s">
-        <v>262</v>
+        <v>246</v>
       </c>
       <c r="I29" s="20"/>
     </row>
@@ -16067,7 +15929,7 @@
       <c r="F30" s="43"/>
       <c r="G30" s="44" t="n">
         <f aca="false">-MOD(G27+G28+G29,1000)</f>
-        <v>-160.987500000745</v>
+        <v>-34.5480000004172</v>
       </c>
       <c r="H30" s="40" t="s">
         <v>247</v>
@@ -16085,7 +15947,7 @@
       <c r="F31" s="45"/>
       <c r="G31" s="46" t="n">
         <f aca="false">G27+G28+G29+G30</f>
-        <v>25653000</v>
+        <v>24747000</v>
       </c>
       <c r="H31" s="10" t="s">
         <v>248</v>
@@ -16219,7 +16081,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="41" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B5" s="41"/>
       <c r="C5" s="41"/>
@@ -16270,7 +16132,7 @@
         <v>180</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E8" s="42" t="n">
         <v>9991</v>
@@ -16283,7 +16145,7 @@
         <v>6993700</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="I8" s="17" t="s">
         <v>69</v>
@@ -16333,7 +16195,7 @@
         <v>160000</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I10" s="17" t="s">
         <v>69</v>
@@ -16387,7 +16249,7 @@
         <v>500000</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I12" s="17" t="s">
         <v>69</v>
@@ -16415,7 +16277,7 @@
         <v>420000</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I13" s="17" t="s">
         <v>69</v>
@@ -16546,7 +16408,7 @@
         <v>202</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E18" s="42" t="n">
         <v>2</v>
@@ -16572,7 +16434,7 @@
         <v>204</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E19" s="42" t="n">
         <v>1</v>
@@ -16611,7 +16473,7 @@
         <v>1200000</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I20" s="17" t="s">
         <v>71</v>
@@ -16667,7 +16529,7 @@
         <v>300000</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I22" s="17" t="s">
         <v>71</v>
@@ -16695,7 +16557,7 @@
         <v>255000</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I23" s="17" t="s">
         <v>71</v>
@@ -16848,10 +16710,10 @@
       <c r="F32" s="43"/>
       <c r="G32" s="44" t="n">
         <f aca="false">(G25+G26+G27+G28+G29+G31)*요율근거!$C$11</f>
-        <v>268813.694205</v>
+        <v>716836.51788</v>
       </c>
       <c r="H32" s="20" t="s">
-        <v>272</v>
+        <v>246</v>
       </c>
       <c r="I32" s="20"/>
     </row>
@@ -16866,7 +16728,7 @@
       <c r="F33" s="43"/>
       <c r="G33" s="44" t="n">
         <f aca="false">-MOD(G30+G31+G32,1000)</f>
-        <v>-970.167704999447</v>
+        <v>-992.991379998624</v>
       </c>
       <c r="H33" s="40" t="s">
         <v>247</v>
@@ -16884,7 +16746,7 @@
       <c r="F34" s="45"/>
       <c r="G34" s="46" t="n">
         <f aca="false">G30+G31+G32+G33</f>
-        <v>18462000</v>
+        <v>18910000</v>
       </c>
       <c r="H34" s="10" t="s">
         <v>248</v>
@@ -16978,24 +16840,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="49" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="C3" s="15" t="s">
         <v>274</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="D3" s="15" t="s">
         <v>275</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="E3" s="15" t="s">
         <v>276</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>277</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17078,7 +16940,7 @@
         <v>88</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>36</v>
@@ -17086,7 +16948,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="56" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B10" s="57" t="n">
         <v>13575440</v>
@@ -17096,12 +16958,12 @@
         <v>1358.73969092802</v>
       </c>
       <c r="D10" s="56" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="56" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B11" s="57" t="n">
         <v>9577783</v>
@@ -17111,12 +16973,12 @@
         <v>958.621887260789</v>
       </c>
       <c r="D11" s="56" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="56" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B12" s="57" t="n">
         <v>4000000</v>
@@ -17126,12 +16988,12 @@
         <v>400.352310032829</v>
       </c>
       <c r="D12" s="56" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="56" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B13" s="58" t="n">
         <f aca="false">E7*700</f>
@@ -17142,12 +17004,12 @@
         <v>700</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="56" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B14" s="58" t="n">
         <f aca="false">B13-(B11-B12)</f>
@@ -17158,12 +17020,12 @@
         <v>141.730422772039</v>
       </c>
       <c r="D14" s="56" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="36" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
   </sheetData>
@@ -17192,56 +17054,56 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="35" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="54" t="s">
+        <v>289</v>
+      </c>
+      <c r="B3" s="54" t="s">
+        <v>290</v>
+      </c>
+      <c r="C3" s="59" t="s">
         <v>291</v>
       </c>
-      <c r="B3" s="54" t="s">
+      <c r="D3" s="59" t="s">
         <v>292</v>
       </c>
-      <c r="C3" s="59" t="s">
+      <c r="E3" s="59" t="s">
         <v>293</v>
       </c>
-      <c r="D3" s="59" t="s">
+      <c r="F3" s="59" t="s">
         <v>294</v>
       </c>
-      <c r="E3" s="59" t="s">
+      <c r="G3" s="59" t="s">
         <v>295</v>
       </c>
-      <c r="F3" s="59" t="s">
+      <c r="H3" s="59" t="s">
         <v>296</v>
       </c>
-      <c r="G3" s="59" t="s">
+      <c r="I3" s="59" t="s">
         <v>297</v>
       </c>
-      <c r="H3" s="59" t="s">
+      <c r="J3" s="59" t="s">
         <v>298</v>
       </c>
-      <c r="I3" s="59" t="s">
+      <c r="K3" s="59" t="s">
         <v>299</v>
       </c>
-      <c r="J3" s="59" t="s">
+      <c r="L3" s="59" t="s">
         <v>300</v>
       </c>
-      <c r="K3" s="59" t="s">
+      <c r="M3" s="59" t="s">
         <v>301</v>
-      </c>
-      <c r="L3" s="59" t="s">
-        <v>302</v>
-      </c>
-      <c r="M3" s="59" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="60" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B4" s="60" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C4" s="61"/>
       <c r="D4" s="56"/>
@@ -17257,10 +17119,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="60" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B5" s="60" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C5" s="61"/>
       <c r="D5" s="61"/>
@@ -17276,10 +17138,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="60" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B6" s="60" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C6" s="56"/>
       <c r="D6" s="56"/>
@@ -17295,10 +17157,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="60" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B7" s="60" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C7" s="56"/>
       <c r="D7" s="56"/>
@@ -17314,10 +17176,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="60" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B8" s="60" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C8" s="56"/>
       <c r="D8" s="56"/>
@@ -17333,10 +17195,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="60" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B9" s="60" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C9" s="56"/>
       <c r="D9" s="56"/>
@@ -17352,10 +17214,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="60" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B10" s="60" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C10" s="56"/>
       <c r="D10" s="56"/>
@@ -17371,7 +17233,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="36" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
   </sheetData>
@@ -17402,26 +17264,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="35" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="36" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
+        <v>318</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>319</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>320</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="D4" s="15" t="s">
         <v>321</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>322</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17429,13 +17291,13 @@
         <v>72</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C5" s="62" t="n">
         <v>0.0356</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17443,13 +17305,13 @@
         <v>73</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C6" s="62" t="n">
         <v>0.0115</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17457,13 +17319,13 @@
         <v>74</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C7" s="62" t="n">
         <v>0.0311</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17471,91 +17333,91 @@
         <v>76</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C8" s="62" t="n">
         <v>0.05</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="C9" s="63" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>331</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>332</v>
-      </c>
-      <c r="C9" s="63" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C10" s="63" t="n">
-        <v>0.125</v>
+        <v>0.08</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C11" s="63" t="n">
-        <v>0.03</v>
+        <v>0.08</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
+        <v>334</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>335</v>
+      </c>
+      <c r="C12" s="16" t="s">
         <v>336</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="D12" s="4" t="s">
         <v>337</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>338</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="64" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
+        <v>339</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>340</v>
+      </c>
+      <c r="C15" s="15" t="s">
         <v>341</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="D15" s="15" t="s">
         <v>342</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="E15" s="15" t="s">
         <v>343</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>344</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17563,7 +17425,7 @@
         <v>144</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C16" s="42" t="n">
         <v>292640</v>
@@ -17578,10 +17440,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C17" s="42" t="n">
         <v>266029</v>
@@ -17599,7 +17461,7 @@
         <v>153</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C18" s="42" t="n">
         <v>226122</v>
@@ -17617,7 +17479,7 @@
         <v>126</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C19" s="42" t="n">
         <v>172068</v>
@@ -17635,7 +17497,7 @@
         <v>159</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C20" s="42" t="n">
         <v>226122</v>
@@ -17653,7 +17515,7 @@
         <v>96</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C21" s="42" t="n">
         <v>226122</v>
@@ -17671,7 +17533,7 @@
         <v>91</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C22" s="42" t="n">
         <v>281939</v>
@@ -17686,7 +17548,7 @@
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="34" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B23" s="34"/>
       <c r="C23" s="34"/>
@@ -17695,15 +17557,15 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="64" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="66" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B26" s="67" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C26" s="67"/>
       <c r="D26" s="67"/>
@@ -17711,10 +17573,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="66" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B27" s="67" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C27" s="67"/>
       <c r="D27" s="67"/>
@@ -17722,10 +17584,10 @@
     </row>
     <row r="28" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="66" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B28" s="67" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C28" s="67"/>
       <c r="D28" s="67"/>
@@ -17736,7 +17598,7 @@
         <v>74</v>
       </c>
       <c r="B29" s="67" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C29" s="67"/>
       <c r="D29" s="67"/>
@@ -17744,10 +17606,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="66" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B30" s="67" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C30" s="67"/>
       <c r="D30" s="67"/>
@@ -17755,10 +17617,10 @@
     </row>
     <row r="31" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="68" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B31" s="67" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C31" s="67"/>
       <c r="D31" s="67"/>
@@ -17766,10 +17628,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="66" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B32" s="69" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C32" s="69"/>
       <c r="D32" s="69"/>
@@ -17777,7 +17639,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="36" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KKT: weights 38t/48t, dates marked as assumed, 200t B-only, right-side elevated view + PiP compose
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014v4o941zghHSMa9tRzfaqP
</commit_message>
<xml_diff>
--- a/experiments/2026-10-12-kkt-drying-furnace-base/estimate/견적서_금강변압기_진공건조로_회전안착_용접_v3.xlsx
+++ b/experiments/2026-10-12-kkt-drying-furnace-base/estimate/견적서_금강변압기_진공건조로_회전안착_용접_v3.xlsx
@@ -452,7 +452,7 @@
     <t xml:space="preserve">특기사항</t>
   </si>
   <si>
-    <t xml:space="preserve">1. 공사 기간: 2026.10.21 ~ 2026.11.02 (가계획, 작업일 11일, 공정표 시트 참조). 착공일은 발주처 협의로 확정함.</t>
+    <t xml:space="preserve">1. 공사 기간: 2026.10.21 ~ 2026.11.02 (가정 일정, 작업일 11일, 공정표 시트 참조). 날짜는 가정이며 착공일은 발주처 협의로 확정함.</t>
   </si>
   <si>
     <t xml:space="preserve">2. 결제 조건: 협의 (예: 착수 30%, 준공 후 70%).</t>
@@ -584,7 +584,7 @@
     <t xml:space="preserve">※ B안 200t급 크레인은 사용자 제시 단가 350만/일 적용. 회송·웨이트 운반은 별도 줄로 넣음. B안 용접은 3면 용접 → 전체 90° 회전 → 나머지 1면 용접 순서로, 용접 1일이 회전 후로 이동함(금액 동일).</t>
   </si>
   <si>
-    <t xml:space="preserve">※ B안 회전은 일체 약 83t(45t + 38t)을 모서리 기준으로 세우는 작업으로, 실제 크레인 사양은 인양계획서·구조검토로 확정 필요함.</t>
+    <t xml:space="preserve">※ B안 회전은 일체 약 86t(38t + 48t)을 모서리 기준으로 세우는 작업으로, 실제 크레인 사양은 인양계획서·구조검토로 확정 필요함.</t>
   </si>
   <si>
     <t xml:space="preserve">※ 회전 후 원래 자세로 되돌리는 회전이나 영구 받침이 필요하면 별도임.</t>
@@ -977,7 +977,7 @@
     <t xml:space="preserve">안착일</t>
   </si>
   <si>
-    <t xml:space="preserve">회전일, 일체 약 83t</t>
+    <t xml:space="preserve">회전일, 일체 약 86t</t>
   </si>
   <si>
     <t xml:space="preserve">대형 크레인 부대비</t>
@@ -1219,7 +1219,7 @@
     <t xml:space="preserve">단위중량 72.4 kg/m는 KS H-250×250×9×14 공칭값임. 베이스는 임시 구조물로 방청·도장 미적용.</t>
   </si>
   <si>
-    <t xml:space="preserve">공정표 (가계획 2026.10.21 ~ 11.02, 작업일 11일)</t>
+    <t xml:space="preserve">공정표 (가정 일정 2026.10.21 ~ 11.02, 작업일 11일)</t>
   </si>
   <si>
     <t xml:space="preserve">공정</t>
@@ -1311,7 +1311,7 @@
     <t xml:space="preserve">펜스 해체·정리</t>
   </si>
   <si>
-    <t xml:space="preserve">가계획: 2026-10-21(수) 착공 ~ 11-02(월) 완료, 일요일 휴무 기준 작업일 11일. 착공일은 발주처 협의로 확정함.</t>
+    <t xml:space="preserve">가정 일정: 2026-10-21(수) 착공 ~ 11-02(월) 완료, 일요일 휴무 기준 작업일 11일. 날짜는 가정이며 착공일은 발주처 협의로 확정함.</t>
   </si>
   <si>
     <t xml:space="preserve">요율 및 단가 근거</t>

</xml_diff>

<commit_message>
KKT quote: payment terms 30/30/40, crane note without ground review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014v4o941zghHSMa9tRzfaqP
</commit_message>
<xml_diff>
--- a/experiments/2026-10-12-kkt-drying-furnace-base/estimate/견적서_금강변압기_진공건조로_회전안착_용접_v3.xlsx
+++ b/experiments/2026-10-12-kkt-drying-furnace-base/estimate/견적서_금강변압기_진공건조로_회전안착_용접_v3.xlsx
@@ -455,7 +455,7 @@
     <t xml:space="preserve">1. 공사 기간: 2026.10.21 ~ 2026.11.02 (가정 일정, 작업일 11일, 공정표 시트 참조). 날짜는 가정이며 착공일은 발주처 협의로 확정함.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. 결제 조건: 협의 (예: 착수 30%, 준공 후 70%).</t>
+    <t xml:space="preserve">2. 결제 조건: 선수금 30% (계약 시), 중도금 30% (회전·안착 완료 시), 잔금 40% (용접 완료 후). A안 VAT 포함 기준 23,658,360원 / 23,658,360원 / 31,544,480원.</t>
   </si>
   <si>
     <t xml:space="preserve">3. 견적 유효기간: 발행일로부터 30일.</t>
@@ -467,7 +467,7 @@
     <t xml:space="preserve">5. 제외: 전기 수전, 배관·닥트 해체·복구, 보온, 도장, 비파괴검사(PT/UT), 시운전. 비파괴검사는 발주처 요구 시 별도 정산함.</t>
   </si>
   <si>
-    <t xml:space="preserve">6. 크레인 사양·배치는 인양계획서와 지반 검토 후 확정하며, 크레인 변경에 따른 추가비용은 없음.</t>
+    <t xml:space="preserve">6. 크레인 사양·배치는 크레인 업체와 협의해 확정하며, 크레인 변경에 따른 추가비용은 없음.</t>
   </si>
   <si>
     <t xml:space="preserve">7. 연장·야간·휴일 작업은 공정에 따라 당사가 수행하며 추가 정산하지 않음. 기상(우천 시 용접 불가)·발주처 사유에 따른 대기는 별도 협의함.</t>
@@ -3883,7 +3883,7 @@
       <c r="H69" s="24"/>
       <c r="I69" s="24"/>
     </row>
-    <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="24" t="s">
         <v>137</v>
       </c>

</xml_diff>